<commit_message>
wrapped up evaluations. used ROUGE, SemScore, and BERTScore to evaluate and create a Composite Score
</commit_message>
<xml_diff>
--- a/project/evaluations/Assistance_Instructions_Bert_Scores.xlsx
+++ b/project/evaluations/Assistance_Instructions_Bert_Scores.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G193"/>
+  <dimension ref="A1:F193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,11 +459,6 @@
           <t>Assistance_Instruction_BERT_F1_Score</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Assistance_Instruction_BLEU_Score</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -490,11 +485,6 @@
       <c r="F2" t="n">
         <v>0.8849157094955444</v>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>BLEU = 0.56 4.4/0.6/0.3/0.1 (BP = 1.000 ratio = 91.000 hyp_len = 91 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -521,11 +511,6 @@
       <c r="F3" t="n">
         <v>0.8824114203453064</v>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>BLEU = 0.56 4.4/0.6/0.3/0.1 (BP = 1.000 ratio = 91.000 hyp_len = 91 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -552,11 +537,6 @@
       <c r="F4" t="n">
         <v>0.8810242414474487</v>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>BLEU = 0.56 4.4/0.6/0.3/0.1 (BP = 1.000 ratio = 91.000 hyp_len = 91 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -583,11 +563,6 @@
       <c r="F5" t="n">
         <v>0.8785361051559448</v>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>BLEU = 0.56 4.4/0.6/0.3/0.1 (BP = 1.000 ratio = 91.000 hyp_len = 91 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -614,11 +589,6 @@
       <c r="F6" t="n">
         <v>0.8792104125022888</v>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>BLEU = 0.56 4.4/0.6/0.3/0.1 (BP = 1.000 ratio = 91.000 hyp_len = 91 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -645,11 +615,6 @@
       <c r="F7" t="n">
         <v>0.8908576369285583</v>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>BLEU = 0.56 4.4/0.6/0.3/0.1 (BP = 1.000 ratio = 91.000 hyp_len = 91 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -676,11 +641,6 @@
       <c r="F8" t="n">
         <v>0.8998137712478638</v>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>BLEU = 0.56 4.4/0.6/0.3/0.1 (BP = 1.000 ratio = 91.000 hyp_len = 91 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -707,11 +667,6 @@
       <c r="F9" t="n">
         <v>0.8841415047645569</v>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>BLEU = 0.56 4.4/0.6/0.3/0.1 (BP = 1.000 ratio = 91.000 hyp_len = 91 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -738,11 +693,6 @@
       <c r="F10" t="n">
         <v>0.8800258636474609</v>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>BLEU = 0.56 4.4/0.6/0.3/0.1 (BP = 1.000 ratio = 91.000 hyp_len = 91 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -769,11 +719,6 @@
       <c r="F11" t="n">
         <v>0.8888394832611084</v>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>BLEU = 0.56 4.4/0.6/0.3/0.1 (BP = 1.000 ratio = 91.000 hyp_len = 91 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -800,11 +745,6 @@
       <c r="F12" t="n">
         <v>0.8825829029083252</v>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>BLEU = 0.56 4.4/0.6/0.3/0.1 (BP = 1.000 ratio = 91.000 hyp_len = 91 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -831,11 +771,6 @@
       <c r="F13" t="n">
         <v>0.8756948113441467</v>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -862,11 +797,6 @@
       <c r="F14" t="n">
         <v>0.8650199174880981</v>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -893,11 +823,6 @@
       <c r="F15" t="n">
         <v>0.8711382150650024</v>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -924,11 +849,6 @@
       <c r="F16" t="n">
         <v>0.878614604473114</v>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -955,11 +875,6 @@
       <c r="F17" t="n">
         <v>0.8800866007804871</v>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -986,11 +901,6 @@
       <c r="F18" t="n">
         <v>0.8733140230178833</v>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1017,11 +927,6 @@
       <c r="F19" t="n">
         <v>0.8794379830360413</v>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1048,11 +953,6 @@
       <c r="F20" t="n">
         <v>0.8771107196807861</v>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1079,11 +979,6 @@
       <c r="F21" t="n">
         <v>0.8709536194801331</v>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1110,11 +1005,6 @@
       <c r="F22" t="n">
         <v>0.8730751872062683</v>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1141,11 +1031,6 @@
       <c r="F23" t="n">
         <v>0.8747912049293518</v>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1172,11 +1057,6 @@
       <c r="F24" t="n">
         <v>0.8678528666496277</v>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1203,11 +1083,6 @@
       <c r="F25" t="n">
         <v>0.8816002011299133</v>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1234,11 +1109,6 @@
       <c r="F26" t="n">
         <v>0.8719335794448853</v>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1265,11 +1135,6 @@
       <c r="F27" t="n">
         <v>0.87247234582901</v>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1296,11 +1161,6 @@
       <c r="F28" t="n">
         <v>0.8715429902076721</v>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1327,11 +1187,6 @@
       <c r="F29" t="n">
         <v>0.8758571147918701</v>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1358,11 +1213,6 @@
       <c r="F30" t="n">
         <v>0.8762255311012268</v>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1389,11 +1239,6 @@
       <c r="F31" t="n">
         <v>0.8781684041023254</v>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1420,11 +1265,6 @@
       <c r="F32" t="n">
         <v>0.8758929967880249</v>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1451,11 +1291,6 @@
       <c r="F33" t="n">
         <v>0.8779250979423523</v>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1482,11 +1317,6 @@
       <c r="F34" t="n">
         <v>0.8744076490402222</v>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1513,11 +1343,6 @@
       <c r="F35" t="n">
         <v>0.8709763288497925</v>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1544,11 +1369,6 @@
       <c r="F36" t="n">
         <v>0.8741331696510315</v>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1575,11 +1395,6 @@
       <c r="F37" t="n">
         <v>0.8809305429458618</v>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1606,11 +1421,6 @@
       <c r="F38" t="n">
         <v>0.8734795451164246</v>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1637,11 +1447,6 @@
       <c r="F39" t="n">
         <v>0.8791655898094177</v>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1668,11 +1473,6 @@
       <c r="F40" t="n">
         <v>0.8771005868911743</v>
       </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1699,11 +1499,6 @@
       <c r="F41" t="n">
         <v>0.8769769072532654</v>
       </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1730,11 +1525,6 @@
       <c r="F42" t="n">
         <v>0.8660303950309753</v>
       </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1761,11 +1551,6 @@
       <c r="F43" t="n">
         <v>0.8754856586456299</v>
       </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1792,11 +1577,6 @@
       <c r="F44" t="n">
         <v>0.861583948135376</v>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1823,11 +1603,6 @@
       <c r="F45" t="n">
         <v>0.8733316659927368</v>
       </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1854,11 +1629,6 @@
       <c r="F46" t="n">
         <v>0.8602023720741272</v>
       </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1885,11 +1655,6 @@
       <c r="F47" t="n">
         <v>0.8691626787185669</v>
       </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1916,11 +1681,6 @@
       <c r="F48" t="n">
         <v>0.8822510242462158</v>
       </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1947,11 +1707,6 @@
       <c r="F49" t="n">
         <v>0.8610090017318726</v>
       </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1978,11 +1733,6 @@
       <c r="F50" t="n">
         <v>0.8724158406257629</v>
       </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2009,11 +1759,6 @@
       <c r="F51" t="n">
         <v>0.86553955078125</v>
       </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2040,11 +1785,6 @@
       <c r="F52" t="n">
         <v>0.8737125992774963</v>
       </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2071,11 +1811,6 @@
       <c r="F53" t="n">
         <v>0.8768825531005859</v>
       </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2102,11 +1837,6 @@
       <c r="F54" t="n">
         <v>0.8685184121131897</v>
       </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2133,11 +1863,6 @@
       <c r="F55" t="n">
         <v>0.8731110095977783</v>
       </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2164,11 +1889,6 @@
       <c r="F56" t="n">
         <v>0.8680337071418762</v>
       </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2195,11 +1915,6 @@
       <c r="F57" t="n">
         <v>0.8734711408615112</v>
       </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2226,11 +1941,6 @@
       <c r="F58" t="n">
         <v>0.8666489124298096</v>
       </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2257,11 +1967,6 @@
       <c r="F59" t="n">
         <v>0.8810017704963684</v>
       </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2288,11 +1993,6 @@
       <c r="F60" t="n">
         <v>0.8736598491668701</v>
       </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2319,11 +2019,6 @@
       <c r="F61" t="n">
         <v>0.8779709935188293</v>
       </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2350,11 +2045,6 @@
       <c r="F62" t="n">
         <v>0.8795854449272156</v>
       </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2381,11 +2071,6 @@
       <c r="F63" t="n">
         <v>0.8695570230484009</v>
       </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2412,11 +2097,6 @@
       <c r="F64" t="n">
         <v>0.8688133955001831</v>
       </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2443,11 +2123,6 @@
       <c r="F65" t="n">
         <v>0.8709536194801331</v>
       </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2474,11 +2149,6 @@
       <c r="F66" t="n">
         <v>0.8642076253890991</v>
       </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2505,11 +2175,6 @@
       <c r="F67" t="n">
         <v>0.8818884491920471</v>
       </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2536,11 +2201,6 @@
       <c r="F68" t="n">
         <v>0.878620445728302</v>
       </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2567,11 +2227,6 @@
       <c r="F69" t="n">
         <v>0.8674899339675903</v>
       </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2598,11 +2253,6 @@
       <c r="F70" t="n">
         <v>0.8775944709777832</v>
       </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2629,11 +2279,6 @@
       <c r="F71" t="n">
         <v>0.8702248930931091</v>
       </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2660,11 +2305,6 @@
       <c r="F72" t="n">
         <v>0.8804507255554199</v>
       </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2691,11 +2331,6 @@
       <c r="F73" t="n">
         <v>0.8784664869308472</v>
       </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2722,11 +2357,6 @@
       <c r="F74" t="n">
         <v>0.8736082911491394</v>
       </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2753,11 +2383,6 @@
       <c r="F75" t="n">
         <v>0.8733260631561279</v>
       </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2784,11 +2409,6 @@
       <c r="F76" t="n">
         <v>0.8812158107757568</v>
       </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2815,11 +2435,6 @@
       <c r="F77" t="n">
         <v>0.8798786997795105</v>
       </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>BLEU = 0.90 5.7/1.0/0.5/0.2 (BP = 1.000 ratio = 53.000 hyp_len = 53 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2846,11 +2461,6 @@
       <c r="F78" t="n">
         <v>0.8395063877105713</v>
       </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>BLEU = 0.40 1.1/0.6/0.3/0.1 (BP = 1.000 ratio = 90.000 hyp_len = 90 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2877,11 +2487,6 @@
       <c r="F79" t="n">
         <v>0.8810881376266479</v>
       </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2908,11 +2513,6 @@
       <c r="F80" t="n">
         <v>0.8746963143348694</v>
       </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2939,11 +2539,6 @@
       <c r="F81" t="n">
         <v>0.8646352887153625</v>
       </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2970,11 +2565,6 @@
       <c r="F82" t="n">
         <v>0.8817905783653259</v>
       </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3001,11 +2591,6 @@
       <c r="F83" t="n">
         <v>0.8723305463790894</v>
       </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3032,11 +2617,6 @@
       <c r="F84" t="n">
         <v>0.8679018616676331</v>
       </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3063,11 +2643,6 @@
       <c r="F85" t="n">
         <v>0.8646030426025391</v>
       </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3094,11 +2669,6 @@
       <c r="F86" t="n">
         <v>0.886121392250061</v>
       </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3125,11 +2695,6 @@
       <c r="F87" t="n">
         <v>0.8681966066360474</v>
       </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3156,11 +2721,6 @@
       <c r="F88" t="n">
         <v>0.8701790571212769</v>
       </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3187,11 +2747,6 @@
       <c r="F89" t="n">
         <v>0.8809128999710083</v>
       </c>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3218,11 +2773,6 @@
       <c r="F90" t="n">
         <v>0.882000207901001</v>
       </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3249,11 +2799,6 @@
       <c r="F91" t="n">
         <v>0.8788173794746399</v>
       </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3280,11 +2825,6 @@
       <c r="F92" t="n">
         <v>0.8678646087646484</v>
       </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3311,11 +2851,6 @@
       <c r="F93" t="n">
         <v>0.8802558779716492</v>
       </c>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3342,11 +2877,6 @@
       <c r="F94" t="n">
         <v>0.8882832527160645</v>
       </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3373,11 +2903,6 @@
       <c r="F95" t="n">
         <v>0.8811932802200317</v>
       </c>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3404,11 +2929,6 @@
       <c r="F96" t="n">
         <v>0.8794350028038025</v>
       </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3435,11 +2955,6 @@
       <c r="F97" t="n">
         <v>0.8772041201591492</v>
       </c>
-      <c r="G97" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3466,11 +2981,6 @@
       <c r="F98" t="n">
         <v>0.8854396939277649</v>
       </c>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3497,11 +3007,6 @@
       <c r="F99" t="n">
         <v>0.8864113092422485</v>
       </c>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3528,11 +3033,6 @@
       <c r="F100" t="n">
         <v>0.8890548944473267</v>
       </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3559,11 +3059,6 @@
       <c r="F101" t="n">
         <v>0.8725852370262146</v>
       </c>
-      <c r="G101" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3590,11 +3085,6 @@
       <c r="F102" t="n">
         <v>0.8777399063110352</v>
       </c>
-      <c r="G102" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3621,11 +3111,6 @@
       <c r="F103" t="n">
         <v>0.877082884311676</v>
       </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>BLEU = 0.78 6.1/0.8/0.4/0.2 (BP = 1.000 ratio = 66.000 hyp_len = 66 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3652,11 +3137,6 @@
       <c r="F104" t="n">
         <v>0.8740279674530029</v>
       </c>
-      <c r="G104" t="inlineStr">
-        <is>
-          <t>BLEU = 0.66 6.1/0.6/0.3/0.2 (BP = 1.000 ratio = 82.000 hyp_len = 82 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -3683,11 +3163,6 @@
       <c r="F105" t="n">
         <v>0.8691301941871643</v>
       </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>BLEU = 0.66 6.1/0.6/0.3/0.2 (BP = 1.000 ratio = 82.000 hyp_len = 82 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -3714,11 +3189,6 @@
       <c r="F106" t="n">
         <v>0.8693456649780273</v>
       </c>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t>BLEU = 0.66 6.1/0.6/0.3/0.2 (BP = 1.000 ratio = 82.000 hyp_len = 82 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -3745,11 +3215,6 @@
       <c r="F107" t="n">
         <v>0.864831268787384</v>
       </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>BLEU = 0.66 6.1/0.6/0.3/0.2 (BP = 1.000 ratio = 82.000 hyp_len = 82 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3776,11 +3241,6 @@
       <c r="F108" t="n">
         <v>0.8711771368980408</v>
       </c>
-      <c r="G108" t="inlineStr">
-        <is>
-          <t>BLEU = 0.66 6.1/0.6/0.3/0.2 (BP = 1.000 ratio = 82.000 hyp_len = 82 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -3807,11 +3267,6 @@
       <c r="F109" t="n">
         <v>0.8694002628326416</v>
       </c>
-      <c r="G109" t="inlineStr">
-        <is>
-          <t>BLEU = 0.66 6.1/0.6/0.3/0.2 (BP = 1.000 ratio = 82.000 hyp_len = 82 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -3838,11 +3293,6 @@
       <c r="F110" t="n">
         <v>0.8640109300613403</v>
       </c>
-      <c r="G110" t="inlineStr">
-        <is>
-          <t>BLEU = 0.66 6.1/0.6/0.3/0.2 (BP = 1.000 ratio = 82.000 hyp_len = 82 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3869,11 +3319,6 @@
       <c r="F111" t="n">
         <v>0.8770714998245239</v>
       </c>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>BLEU = 0.66 6.1/0.6/0.3/0.2 (BP = 1.000 ratio = 82.000 hyp_len = 82 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3900,11 +3345,6 @@
       <c r="F112" t="n">
         <v>0.8726363778114319</v>
       </c>
-      <c r="G112" t="inlineStr">
-        <is>
-          <t>BLEU = 0.66 6.1/0.6/0.3/0.2 (BP = 1.000 ratio = 82.000 hyp_len = 82 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3931,11 +3371,6 @@
       <c r="F113" t="n">
         <v>0.8647041916847229</v>
       </c>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>BLEU = 0.66 6.1/0.6/0.3/0.2 (BP = 1.000 ratio = 82.000 hyp_len = 82 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3962,11 +3397,6 @@
       <c r="F114" t="n">
         <v>0.9026371836662292</v>
       </c>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>BLEU = 0.87 6.8/0.9/0.4/0.2 (BP = 1.000 ratio = 59.000 hyp_len = 59 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3993,11 +3423,6 @@
       <c r="F115" t="n">
         <v>0.898335337638855</v>
       </c>
-      <c r="G115" t="inlineStr">
-        <is>
-          <t>BLEU = 0.87 6.8/0.9/0.4/0.2 (BP = 1.000 ratio = 59.000 hyp_len = 59 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -4024,11 +3449,6 @@
       <c r="F116" t="n">
         <v>0.9051481485366821</v>
       </c>
-      <c r="G116" t="inlineStr">
-        <is>
-          <t>BLEU = 0.87 6.8/0.9/0.4/0.2 (BP = 1.000 ratio = 59.000 hyp_len = 59 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -4055,11 +3475,6 @@
       <c r="F117" t="n">
         <v>0.9091752171516418</v>
       </c>
-      <c r="G117" t="inlineStr">
-        <is>
-          <t>BLEU = 0.87 6.8/0.9/0.4/0.2 (BP = 1.000 ratio = 59.000 hyp_len = 59 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -4086,11 +3501,6 @@
       <c r="F118" t="n">
         <v>0.9081761240959167</v>
       </c>
-      <c r="G118" t="inlineStr">
-        <is>
-          <t>BLEU = 0.87 6.8/0.9/0.4/0.2 (BP = 1.000 ratio = 59.000 hyp_len = 59 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -4117,11 +3527,6 @@
       <c r="F119" t="n">
         <v>0.8989189863204956</v>
       </c>
-      <c r="G119" t="inlineStr">
-        <is>
-          <t>BLEU = 0.87 6.8/0.9/0.4/0.2 (BP = 1.000 ratio = 59.000 hyp_len = 59 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -4148,11 +3553,6 @@
       <c r="F120" t="n">
         <v>0.9021960496902466</v>
       </c>
-      <c r="G120" t="inlineStr">
-        <is>
-          <t>BLEU = 0.87 6.8/0.9/0.4/0.2 (BP = 1.000 ratio = 59.000 hyp_len = 59 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -4179,11 +3579,6 @@
       <c r="F121" t="n">
         <v>0.9069811701774597</v>
       </c>
-      <c r="G121" t="inlineStr">
-        <is>
-          <t>BLEU = 0.87 6.8/0.9/0.4/0.2 (BP = 1.000 ratio = 59.000 hyp_len = 59 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -4210,11 +3605,6 @@
       <c r="F122" t="n">
         <v>0.903861403465271</v>
       </c>
-      <c r="G122" t="inlineStr">
-        <is>
-          <t>BLEU = 0.87 6.8/0.9/0.4/0.2 (BP = 1.000 ratio = 59.000 hyp_len = 59 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4241,11 +3631,6 @@
       <c r="F123" t="n">
         <v>0.9120023250579834</v>
       </c>
-      <c r="G123" t="inlineStr">
-        <is>
-          <t>BLEU = 0.87 6.8/0.9/0.4/0.2 (BP = 1.000 ratio = 59.000 hyp_len = 59 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4272,11 +3657,6 @@
       <c r="F124" t="n">
         <v>0.902279794216156</v>
       </c>
-      <c r="G124" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 4.5/0.6/0.3/0.1 (BP = 1.000 ratio = 88.000 hyp_len = 88 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -4303,11 +3683,6 @@
       <c r="F125" t="n">
         <v>0.8956314325332642</v>
       </c>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 4.5/0.6/0.3/0.1 (BP = 1.000 ratio = 88.000 hyp_len = 88 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -4334,11 +3709,6 @@
       <c r="F126" t="n">
         <v>0.8911066651344299</v>
       </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 4.5/0.6/0.3/0.1 (BP = 1.000 ratio = 88.000 hyp_len = 88 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -4365,11 +3735,6 @@
       <c r="F127" t="n">
         <v>0.9064555764198303</v>
       </c>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 4.5/0.6/0.3/0.1 (BP = 1.000 ratio = 88.000 hyp_len = 88 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4396,11 +3761,6 @@
       <c r="F128" t="n">
         <v>0.8938810229301453</v>
       </c>
-      <c r="G128" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 4.5/0.6/0.3/0.1 (BP = 1.000 ratio = 88.000 hyp_len = 88 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4427,11 +3787,6 @@
       <c r="F129" t="n">
         <v>0.8895229697227478</v>
       </c>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 4.5/0.6/0.3/0.1 (BP = 1.000 ratio = 88.000 hyp_len = 88 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -4458,11 +3813,6 @@
       <c r="F130" t="n">
         <v>0.8954483866691589</v>
       </c>
-      <c r="G130" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 4.5/0.6/0.3/0.1 (BP = 1.000 ratio = 88.000 hyp_len = 88 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4489,11 +3839,6 @@
       <c r="F131" t="n">
         <v>0.8925533890724182</v>
       </c>
-      <c r="G131" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 4.5/0.6/0.3/0.1 (BP = 1.000 ratio = 88.000 hyp_len = 88 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4520,11 +3865,6 @@
       <c r="F132" t="n">
         <v>0.8957626223564148</v>
       </c>
-      <c r="G132" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 4.5/0.6/0.3/0.1 (BP = 1.000 ratio = 88.000 hyp_len = 88 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4551,11 +3891,6 @@
       <c r="F133" t="n">
         <v>0.8832512497901917</v>
       </c>
-      <c r="G133" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 4.5/0.6/0.3/0.1 (BP = 1.000 ratio = 88.000 hyp_len = 88 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4582,11 +3917,6 @@
       <c r="F134" t="n">
         <v>0.8790066838264465</v>
       </c>
-      <c r="G134" t="inlineStr">
-        <is>
-          <t>BLEU = 0.67 6.2/0.6/0.3/0.2 (BP = 1.000 ratio = 81.000 hyp_len = 81 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4613,11 +3943,6 @@
       <c r="F135" t="n">
         <v>0.8835106492042542</v>
       </c>
-      <c r="G135" t="inlineStr">
-        <is>
-          <t>BLEU = 0.67 6.2/0.6/0.3/0.2 (BP = 1.000 ratio = 81.000 hyp_len = 81 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -4644,11 +3969,6 @@
       <c r="F136" t="n">
         <v>0.8961349129676819</v>
       </c>
-      <c r="G136" t="inlineStr">
-        <is>
-          <t>BLEU = 0.67 6.2/0.6/0.3/0.2 (BP = 1.000 ratio = 81.000 hyp_len = 81 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -4675,11 +3995,6 @@
       <c r="F137" t="n">
         <v>0.8803220391273499</v>
       </c>
-      <c r="G137" t="inlineStr">
-        <is>
-          <t>BLEU = 0.67 6.2/0.6/0.3/0.2 (BP = 1.000 ratio = 81.000 hyp_len = 81 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -4706,11 +4021,6 @@
       <c r="F138" t="n">
         <v>0.8806105256080627</v>
       </c>
-      <c r="G138" t="inlineStr">
-        <is>
-          <t>BLEU = 0.67 6.2/0.6/0.3/0.2 (BP = 1.000 ratio = 81.000 hyp_len = 81 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -4737,11 +4047,6 @@
       <c r="F139" t="n">
         <v>0.8763676881790161</v>
       </c>
-      <c r="G139" t="inlineStr">
-        <is>
-          <t>BLEU = 0.67 6.2/0.6/0.3/0.2 (BP = 1.000 ratio = 81.000 hyp_len = 81 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -4768,11 +4073,6 @@
       <c r="F140" t="n">
         <v>0.8789765238761902</v>
       </c>
-      <c r="G140" t="inlineStr">
-        <is>
-          <t>BLEU = 0.67 6.2/0.6/0.3/0.2 (BP = 1.000 ratio = 81.000 hyp_len = 81 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -4799,11 +4099,6 @@
       <c r="F141" t="n">
         <v>0.8838959336280823</v>
       </c>
-      <c r="G141" t="inlineStr">
-        <is>
-          <t>BLEU = 0.67 6.2/0.6/0.3/0.2 (BP = 1.000 ratio = 81.000 hyp_len = 81 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -4830,11 +4125,6 @@
       <c r="F142" t="n">
         <v>0.8905531764030457</v>
       </c>
-      <c r="G142" t="inlineStr">
-        <is>
-          <t>BLEU = 0.67 6.2/0.6/0.3/0.2 (BP = 1.000 ratio = 81.000 hyp_len = 81 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -4861,11 +4151,6 @@
       <c r="F143" t="n">
         <v>0.8856889605522156</v>
       </c>
-      <c r="G143" t="inlineStr">
-        <is>
-          <t>BLEU = 0.67 6.2/0.6/0.3/0.2 (BP = 1.000 ratio = 81.000 hyp_len = 81 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -4892,11 +4177,6 @@
       <c r="F144" t="n">
         <v>0.88683021068573</v>
       </c>
-      <c r="G144" t="inlineStr">
-        <is>
-          <t>BLEU = 0.70 6.5/0.7/0.3/0.2 (BP = 1.000 ratio = 77.000 hyp_len = 77 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -4923,11 +4203,6 @@
       <c r="F145" t="n">
         <v>0.8848605751991272</v>
       </c>
-      <c r="G145" t="inlineStr">
-        <is>
-          <t>BLEU = 0.70 6.5/0.7/0.3/0.2 (BP = 1.000 ratio = 77.000 hyp_len = 77 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -4954,11 +4229,6 @@
       <c r="F146" t="n">
         <v>0.8828306794166565</v>
       </c>
-      <c r="G146" t="inlineStr">
-        <is>
-          <t>BLEU = 0.70 6.5/0.7/0.3/0.2 (BP = 1.000 ratio = 77.000 hyp_len = 77 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -4985,11 +4255,6 @@
       <c r="F147" t="n">
         <v>0.8902860283851624</v>
       </c>
-      <c r="G147" t="inlineStr">
-        <is>
-          <t>BLEU = 0.70 6.5/0.7/0.3/0.2 (BP = 1.000 ratio = 77.000 hyp_len = 77 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -5016,11 +4281,6 @@
       <c r="F148" t="n">
         <v>0.8875819444656372</v>
       </c>
-      <c r="G148" t="inlineStr">
-        <is>
-          <t>BLEU = 0.70 6.5/0.7/0.3/0.2 (BP = 1.000 ratio = 77.000 hyp_len = 77 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -5047,11 +4307,6 @@
       <c r="F149" t="n">
         <v>0.88753741979599</v>
       </c>
-      <c r="G149" t="inlineStr">
-        <is>
-          <t>BLEU = 0.70 6.5/0.7/0.3/0.2 (BP = 1.000 ratio = 77.000 hyp_len = 77 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -5078,11 +4333,6 @@
       <c r="F150" t="n">
         <v>0.8808034062385559</v>
       </c>
-      <c r="G150" t="inlineStr">
-        <is>
-          <t>BLEU = 0.70 6.5/0.7/0.3/0.2 (BP = 1.000 ratio = 77.000 hyp_len = 77 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -5109,11 +4359,6 @@
       <c r="F151" t="n">
         <v>0.8779293894767761</v>
       </c>
-      <c r="G151" t="inlineStr">
-        <is>
-          <t>BLEU = 0.70 6.5/0.7/0.3/0.2 (BP = 1.000 ratio = 77.000 hyp_len = 77 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -5140,11 +4385,6 @@
       <c r="F152" t="n">
         <v>0.8883615136146545</v>
       </c>
-      <c r="G152" t="inlineStr">
-        <is>
-          <t>BLEU = 0.70 6.5/0.7/0.3/0.2 (BP = 1.000 ratio = 77.000 hyp_len = 77 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -5171,11 +4411,6 @@
       <c r="F153" t="n">
         <v>0.8747519850730896</v>
       </c>
-      <c r="G153" t="inlineStr">
-        <is>
-          <t>BLEU = 0.70 6.5/0.7/0.3/0.2 (BP = 1.000 ratio = 77.000 hyp_len = 77 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -5202,11 +4437,6 @@
       <c r="F154" t="n">
         <v>0.8818499445915222</v>
       </c>
-      <c r="G154" t="inlineStr">
-        <is>
-          <t>BLEU = 0.51 4.7/0.5/0.2/0.1 (BP = 1.000 ratio = 106.000 hyp_len = 106 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -5233,11 +4463,6 @@
       <c r="F155" t="n">
         <v>0.879934549331665</v>
       </c>
-      <c r="G155" t="inlineStr">
-        <is>
-          <t>BLEU = 0.51 4.7/0.5/0.2/0.1 (BP = 1.000 ratio = 106.000 hyp_len = 106 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -5264,11 +4489,6 @@
       <c r="F156" t="n">
         <v>0.8811904191970825</v>
       </c>
-      <c r="G156" t="inlineStr">
-        <is>
-          <t>BLEU = 0.51 4.7/0.5/0.2/0.1 (BP = 1.000 ratio = 106.000 hyp_len = 106 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -5295,11 +4515,6 @@
       <c r="F157" t="n">
         <v>0.8742616772651672</v>
       </c>
-      <c r="G157" t="inlineStr">
-        <is>
-          <t>BLEU = 0.51 4.7/0.5/0.2/0.1 (BP = 1.000 ratio = 106.000 hyp_len = 106 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -5326,11 +4541,6 @@
       <c r="F158" t="n">
         <v>0.8860466480255127</v>
       </c>
-      <c r="G158" t="inlineStr">
-        <is>
-          <t>BLEU = 0.51 4.7/0.5/0.2/0.1 (BP = 1.000 ratio = 106.000 hyp_len = 106 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -5357,11 +4567,6 @@
       <c r="F159" t="n">
         <v>0.878786027431488</v>
       </c>
-      <c r="G159" t="inlineStr">
-        <is>
-          <t>BLEU = 0.51 4.7/0.5/0.2/0.1 (BP = 1.000 ratio = 106.000 hyp_len = 106 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -5388,11 +4593,6 @@
       <c r="F160" t="n">
         <v>0.8824982643127441</v>
       </c>
-      <c r="G160" t="inlineStr">
-        <is>
-          <t>BLEU = 0.51 4.7/0.5/0.2/0.1 (BP = 1.000 ratio = 106.000 hyp_len = 106 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -5419,11 +4619,6 @@
       <c r="F161" t="n">
         <v>0.8810548782348633</v>
       </c>
-      <c r="G161" t="inlineStr">
-        <is>
-          <t>BLEU = 0.51 4.7/0.5/0.2/0.1 (BP = 1.000 ratio = 106.000 hyp_len = 106 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -5450,11 +4645,6 @@
       <c r="F162" t="n">
         <v>0.8789445161819458</v>
       </c>
-      <c r="G162" t="inlineStr">
-        <is>
-          <t>BLEU = 0.51 4.7/0.5/0.2/0.1 (BP = 1.000 ratio = 106.000 hyp_len = 106 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -5481,11 +4671,6 @@
       <c r="F163" t="n">
         <v>0.8904046416282654</v>
       </c>
-      <c r="G163" t="inlineStr">
-        <is>
-          <t>BLEU = 0.51 4.7/0.5/0.2/0.1 (BP = 1.000 ratio = 106.000 hyp_len = 106 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -5512,11 +4697,6 @@
       <c r="F164" t="n">
         <v>0.8908814191818237</v>
       </c>
-      <c r="G164" t="inlineStr">
-        <is>
-          <t>BLEU = 0.69 6.4/0.6/0.3/0.2 (BP = 1.000 ratio = 78.000 hyp_len = 78 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -5543,11 +4723,6 @@
       <c r="F165" t="n">
         <v>0.882070779800415</v>
       </c>
-      <c r="G165" t="inlineStr">
-        <is>
-          <t>BLEU = 0.69 6.4/0.6/0.3/0.2 (BP = 1.000 ratio = 78.000 hyp_len = 78 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -5574,11 +4749,6 @@
       <c r="F166" t="n">
         <v>0.898029625415802</v>
       </c>
-      <c r="G166" t="inlineStr">
-        <is>
-          <t>BLEU = 0.69 6.4/0.6/0.3/0.2 (BP = 1.000 ratio = 78.000 hyp_len = 78 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -5605,11 +4775,6 @@
       <c r="F167" t="n">
         <v>0.896388828754425</v>
       </c>
-      <c r="G167" t="inlineStr">
-        <is>
-          <t>BLEU = 0.69 6.4/0.6/0.3/0.2 (BP = 1.000 ratio = 78.000 hyp_len = 78 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -5636,11 +4801,6 @@
       <c r="F168" t="n">
         <v>0.8735437989234924</v>
       </c>
-      <c r="G168" t="inlineStr">
-        <is>
-          <t>BLEU = 0.69 6.4/0.6/0.3/0.2 (BP = 1.000 ratio = 78.000 hyp_len = 78 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -5668,11 +4828,6 @@
       <c r="F169" t="n">
         <v>0.8798334002494812</v>
       </c>
-      <c r="G169" t="inlineStr">
-        <is>
-          <t>BLEU = 0.69 6.4/0.6/0.3/0.2 (BP = 1.000 ratio = 78.000 hyp_len = 78 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -5699,11 +4854,6 @@
       <c r="F170" t="n">
         <v>0.902393639087677</v>
       </c>
-      <c r="G170" t="inlineStr">
-        <is>
-          <t>BLEU = 0.69 6.4/0.6/0.3/0.2 (BP = 1.000 ratio = 78.000 hyp_len = 78 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -5730,11 +4880,6 @@
       <c r="F171" t="n">
         <v>0.8979891538619995</v>
       </c>
-      <c r="G171" t="inlineStr">
-        <is>
-          <t>BLEU = 0.69 6.4/0.6/0.3/0.2 (BP = 1.000 ratio = 78.000 hyp_len = 78 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -5761,11 +4906,6 @@
       <c r="F172" t="n">
         <v>0.8881901502609253</v>
       </c>
-      <c r="G172" t="inlineStr">
-        <is>
-          <t>BLEU = 0.69 6.4/0.6/0.3/0.2 (BP = 1.000 ratio = 78.000 hyp_len = 78 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -5793,11 +4933,6 @@
       <c r="F173" t="n">
         <v>0.8866750001907349</v>
       </c>
-      <c r="G173" t="inlineStr">
-        <is>
-          <t>BLEU = 0.69 6.4/0.6/0.3/0.2 (BP = 1.000 ratio = 78.000 hyp_len = 78 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -5807,7 +4942,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>3. Assistance needed: First respondered should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
+          <t>3. Assistance needed: First responders should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -5816,18 +4951,13 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>0.8578058481216431</v>
+        <v>0.8609910607337952</v>
       </c>
       <c r="E174" t="n">
-        <v>0.909643292427063</v>
+        <v>0.9155696034431458</v>
       </c>
       <c r="F174" t="n">
-        <v>0.8829644322395325</v>
-      </c>
-      <c r="G174" t="inlineStr">
-        <is>
-          <t>BLEU = 0.50 4.6/0.5/0.2/0.1 (BP = 1.000 ratio = 108.000 hyp_len = 108 ref_len = 1)</t>
-        </is>
+        <v>0.8874419331550598</v>
       </c>
     </row>
     <row r="175">
@@ -5838,7 +4968,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>3. Assistance needed: First respondered should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
+          <t>3. Assistance needed: First responders should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -5847,18 +4977,13 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>0.8829092979431152</v>
+        <v>0.8848273754119873</v>
       </c>
       <c r="E175" t="n">
-        <v>0.9007253050804138</v>
+        <v>0.907776415348053</v>
       </c>
       <c r="F175" t="n">
-        <v>0.8917282819747925</v>
-      </c>
-      <c r="G175" t="inlineStr">
-        <is>
-          <t>BLEU = 0.50 4.6/0.5/0.2/0.1 (BP = 1.000 ratio = 108.000 hyp_len = 108 ref_len = 1)</t>
-        </is>
+        <v>0.8961549997329712</v>
       </c>
     </row>
     <row r="176">
@@ -5869,7 +4994,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>3. Assistance needed: First respondered should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
+          <t>3. Assistance needed: First responders should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -5878,18 +5003,13 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>0.8487586975097656</v>
+        <v>0.8500748872756958</v>
       </c>
       <c r="E176" t="n">
-        <v>0.9081562757492065</v>
+        <v>0.9127408862113953</v>
       </c>
       <c r="F176" t="n">
-        <v>0.8774534463882446</v>
-      </c>
-      <c r="G176" t="inlineStr">
-        <is>
-          <t>BLEU = 0.50 4.6/0.5/0.2/0.1 (BP = 1.000 ratio = 108.000 hyp_len = 108 ref_len = 1)</t>
-        </is>
+        <v>0.8802940845489502</v>
       </c>
     </row>
     <row r="177">
@@ -5900,7 +5020,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>3. Assistance needed: First respondered should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
+          <t>3. Assistance needed: First responders should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -5909,18 +5029,13 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>0.8580312728881836</v>
+        <v>0.8597216010093689</v>
       </c>
       <c r="E177" t="n">
-        <v>0.9075081944465637</v>
+        <v>0.9149205684661865</v>
       </c>
       <c r="F177" t="n">
-        <v>0.8820765018463135</v>
-      </c>
-      <c r="G177" t="inlineStr">
-        <is>
-          <t>BLEU = 0.50 4.6/0.5/0.2/0.1 (BP = 1.000 ratio = 108.000 hyp_len = 108 ref_len = 1)</t>
-        </is>
+        <v>0.8864626288414001</v>
       </c>
     </row>
     <row r="178">
@@ -5931,7 +5046,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>3. Assistance needed: First respondered should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
+          <t>3. Assistance needed: First responders should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -5940,18 +5055,13 @@
         </is>
       </c>
       <c r="D178" t="n">
-        <v>0.8423901796340942</v>
+        <v>0.8447442054748535</v>
       </c>
       <c r="E178" t="n">
-        <v>0.9029071927070618</v>
+        <v>0.9119502305984497</v>
       </c>
       <c r="F178" t="n">
-        <v>0.8715994358062744</v>
-      </c>
-      <c r="G178" t="inlineStr">
-        <is>
-          <t>BLEU = 0.50 4.6/0.5/0.2/0.1 (BP = 1.000 ratio = 108.000 hyp_len = 108 ref_len = 1)</t>
-        </is>
+        <v>0.8770617246627808</v>
       </c>
     </row>
     <row r="179">
@@ -5962,7 +5072,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>3. Assistance needed: First respondered should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
+          <t>3. Assistance needed: First responders should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -5971,18 +5081,13 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>0.8498966693878174</v>
+        <v>0.8506507873535156</v>
       </c>
       <c r="E179" t="n">
-        <v>0.9044119119644165</v>
+        <v>0.9117698669433594</v>
       </c>
       <c r="F179" t="n">
-        <v>0.8763072490692139</v>
-      </c>
-      <c r="G179" t="inlineStr">
-        <is>
-          <t>BLEU = 0.50 4.6/0.5/0.2/0.1 (BP = 1.000 ratio = 108.000 hyp_len = 108 ref_len = 1)</t>
-        </is>
+        <v>0.8801505565643311</v>
       </c>
     </row>
     <row r="180">
@@ -5993,7 +5098,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>3. Assistance needed: First respondered should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
+          <t>3. Assistance needed: First responders should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -6002,18 +5107,13 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>0.8518341779708862</v>
+        <v>0.8543193340301514</v>
       </c>
       <c r="E180" t="n">
-        <v>0.9128623604774475</v>
+        <v>0.9183194637298584</v>
       </c>
       <c r="F180" t="n">
-        <v>0.881292998790741</v>
-      </c>
-      <c r="G180" t="inlineStr">
-        <is>
-          <t>BLEU = 0.50 4.6/0.5/0.2/0.1 (BP = 1.000 ratio = 108.000 hyp_len = 108 ref_len = 1)</t>
-        </is>
+        <v>0.8851640820503235</v>
       </c>
     </row>
     <row r="181">
@@ -6024,7 +5124,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>3. Assistance needed: First respondered should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
+          <t>3. Assistance needed: First responders should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -6033,18 +5133,13 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>0.8395174145698547</v>
+        <v>0.8422259092330933</v>
       </c>
       <c r="E181" t="n">
-        <v>0.8831619024276733</v>
+        <v>0.8898535966873169</v>
       </c>
       <c r="F181" t="n">
-        <v>0.8607867956161499</v>
-      </c>
-      <c r="G181" t="inlineStr">
-        <is>
-          <t>BLEU = 0.50 4.6/0.5/0.2/0.1 (BP = 1.000 ratio = 108.000 hyp_len = 108 ref_len = 1)</t>
-        </is>
+        <v>0.8653849363327026</v>
       </c>
     </row>
     <row r="182">
@@ -6055,7 +5150,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>3. Assistance needed: First respondered should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
+          <t>3. Assistance needed: First responders should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -6064,18 +5159,13 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>0.8331766724586487</v>
+        <v>0.8343950510025024</v>
       </c>
       <c r="E182" t="n">
-        <v>0.8923373818397522</v>
+        <v>0.9005779027938843</v>
       </c>
       <c r="F182" t="n">
-        <v>0.8617427945137024</v>
-      </c>
-      <c r="G182" t="inlineStr">
-        <is>
-          <t>BLEU = 0.50 4.6/0.5/0.2/0.1 (BP = 1.000 ratio = 108.000 hyp_len = 108 ref_len = 1)</t>
-        </is>
+        <v>0.8662241101264954</v>
       </c>
     </row>
     <row r="183">
@@ -6086,7 +5176,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>3. Assistance needed: First respondered should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
+          <t>3. Assistance needed: First responders should be deployed immediately to return the man inside the building or provide a surface to catch the man safely.</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -6095,18 +5185,13 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>0.8512947559356689</v>
+        <v>0.8524169921875</v>
       </c>
       <c r="E183" t="n">
-        <v>0.9009701609611511</v>
+        <v>0.9069342613220215</v>
       </c>
       <c r="F183" t="n">
-        <v>0.875428318977356</v>
-      </c>
-      <c r="G183" t="inlineStr">
-        <is>
-          <t>BLEU = 0.50 4.6/0.5/0.2/0.1 (BP = 1.000 ratio = 108.000 hyp_len = 108 ref_len = 1)</t>
-        </is>
+        <v>0.8788309693336487</v>
       </c>
     </row>
     <row r="184">
@@ -6134,11 +5219,6 @@
       <c r="F184" t="n">
         <v>0.9016168117523193</v>
       </c>
-      <c r="G184" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 5.4/0.5/0.3/0.1 (BP = 1.000 ratio = 93.000 hyp_len = 93 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -6165,11 +5245,6 @@
       <c r="F185" t="n">
         <v>0.8881382346153259</v>
       </c>
-      <c r="G185" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 5.4/0.5/0.3/0.1 (BP = 1.000 ratio = 93.000 hyp_len = 93 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -6196,11 +5271,6 @@
       <c r="F186" t="n">
         <v>0.9072278141975403</v>
       </c>
-      <c r="G186" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 5.4/0.5/0.3/0.1 (BP = 1.000 ratio = 93.000 hyp_len = 93 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -6227,11 +5297,6 @@
       <c r="F187" t="n">
         <v>0.8960020542144775</v>
       </c>
-      <c r="G187" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 5.4/0.5/0.3/0.1 (BP = 1.000 ratio = 93.000 hyp_len = 93 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -6258,11 +5323,6 @@
       <c r="F188" t="n">
         <v>0.89410799741745</v>
       </c>
-      <c r="G188" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 5.4/0.5/0.3/0.1 (BP = 1.000 ratio = 93.000 hyp_len = 93 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -6289,11 +5349,6 @@
       <c r="F189" t="n">
         <v>0.8855193257331848</v>
       </c>
-      <c r="G189" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 5.4/0.5/0.3/0.1 (BP = 1.000 ratio = 93.000 hyp_len = 93 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -6320,11 +5375,6 @@
       <c r="F190" t="n">
         <v>0.8899452090263367</v>
       </c>
-      <c r="G190" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 5.4/0.5/0.3/0.1 (BP = 1.000 ratio = 93.000 hyp_len = 93 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -6351,11 +5401,6 @@
       <c r="F191" t="n">
         <v>0.9036219716072083</v>
       </c>
-      <c r="G191" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 5.4/0.5/0.3/0.1 (BP = 1.000 ratio = 93.000 hyp_len = 93 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -6382,11 +5427,6 @@
       <c r="F192" t="n">
         <v>0.9003872275352478</v>
       </c>
-      <c r="G192" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 5.4/0.5/0.3/0.1 (BP = 1.000 ratio = 93.000 hyp_len = 93 ref_len = 1)</t>
-        </is>
-      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -6412,11 +5452,6 @@
       </c>
       <c r="F193" t="n">
         <v>0.8997277617454529</v>
-      </c>
-      <c r="G193" t="inlineStr">
-        <is>
-          <t>BLEU = 0.58 5.4/0.5/0.3/0.1 (BP = 1.000 ratio = 93.000 hyp_len = 93 ref_len = 1)</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>